<commit_message>
Align role titles and experience with CV
Business Analyst titles replace founder titles, MyTicketSeller and NaijaFoodFestival are credited to HunterTV Africa, contract roles are marked, and experience is stated as nine years.
</commit_message>
<xml_diff>
--- a/01-delivered-case-studies/komfort-place-signature-digital-growth/Excel/Project_Workbook.xlsx
+++ b/01-delivered-case-studies/komfort-place-signature-digital-growth/Excel/Project_Workbook.xlsx
@@ -459,6 +459,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="10">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -491,7 +492,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Digital Product Lead and Business Analyst</t>
+          <t>Business Analyst (Contract)</t>
         </is>
       </c>
     </row>
@@ -507,6 +508,8 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="10">
       <c r="A9" s="14" t="inlineStr">
         <is>
@@ -652,6 +655,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="10">
       <c r="A19" s="16" t="inlineStr">
         <is>
@@ -2011,7 +2015,7 @@
       </c>
       <c r="E2" s="18" t="inlineStr">
         <is>
-          <t>Digital product lead</t>
+          <t>Business analyst</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2042,7 @@
       </c>
       <c r="E3" s="18" t="inlineStr">
         <is>
-          <t>Digital product lead</t>
+          <t>Business analyst</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2096,7 @@
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>Digital product lead</t>
+          <t>Business analyst</t>
         </is>
       </c>
     </row>

</xml_diff>